<commit_message>
Se termina modulo Devengado
</commit_message>
<xml_diff>
--- a/public/CuentasCuentas/Rec-CuentasCuentasSeguidas.xlsx
+++ b/public/CuentasCuentas/Rec-CuentasCuentasSeguidas.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RMartinez\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dmijangos\Documents\SAC-IPE\public\Guia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96A1FD22-E234-41A0-A1C5-BEB8DC64E996}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED2C76AD-C482-4C15-9ED6-868B77BF4B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{BA794CD9-A794-4D6D-97A5-04484BD59B08}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BA794CD9-A794-4D6D-97A5-04484BD59B08}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="74">
   <si>
     <t>cuenta</t>
   </si>
@@ -258,12 +259,6 @@
   </si>
   <si>
     <t>II.1.8 PARTICIPACIONES, APORTACIONES, CONVENIOS, INCENTIVOS DERIVADOS DE LA COLABORACIÓN FISCAL, FONDOS DISTINTOS DE APORTACIONES, TRANSFERENCIAS, ASIGNACIONES, SUBSIDIOS Y SUBVENCIONES, Y PENSIONES Y JUBILACIONES</t>
-  </si>
-  <si>
-    <t>Por el recaudo de otros ingresos propios por pensiones.</t>
-  </si>
-  <si>
-    <t>VII.1.1 (OTROS INGRESOS Y BENEFICIOS)</t>
   </si>
 </sst>
 </file>
@@ -1844,10 +1839,10 @@
         <v>32</v>
       </c>
       <c r="B86" t="s">
-        <v>75</v>
-      </c>
-      <c r="C86" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C86" t="s">
+        <v>69</v>
       </c>
       <c r="D86" t="s">
         <v>16</v>
@@ -1858,10 +1853,10 @@
         <v>31</v>
       </c>
       <c r="B87" t="s">
-        <v>75</v>
-      </c>
-      <c r="C87" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C87" t="s">
+        <v>69</v>
       </c>
       <c r="D87" t="s">
         <v>33</v>
@@ -1872,10 +1867,10 @@
         <v>32</v>
       </c>
       <c r="B88" t="s">
-        <v>75</v>
-      </c>
-      <c r="C88" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C88" t="s">
+        <v>69</v>
       </c>
       <c r="D88" t="s">
         <v>16</v>
@@ -1886,10 +1881,10 @@
         <v>49</v>
       </c>
       <c r="B89" t="s">
-        <v>75</v>
-      </c>
-      <c r="C89" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C89" t="s">
+        <v>69</v>
       </c>
       <c r="D89" t="s">
         <v>5</v>
@@ -1900,10 +1895,10 @@
         <v>32</v>
       </c>
       <c r="B90" t="s">
-        <v>75</v>
-      </c>
-      <c r="C90" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C90" t="s">
+        <v>69</v>
       </c>
       <c r="D90" t="s">
         <v>16</v>
@@ -1914,10 +1909,10 @@
         <v>51</v>
       </c>
       <c r="B91" t="s">
-        <v>75</v>
-      </c>
-      <c r="C91" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C91" t="s">
+        <v>69</v>
       </c>
       <c r="D91" t="s">
         <v>34</v>
@@ -1928,10 +1923,10 @@
         <v>32</v>
       </c>
       <c r="B92" t="s">
-        <v>75</v>
-      </c>
-      <c r="C92" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C92" t="s">
+        <v>69</v>
       </c>
       <c r="D92" t="s">
         <v>16</v>
@@ -1942,10 +1937,10 @@
         <v>31</v>
       </c>
       <c r="B93" t="s">
-        <v>75</v>
-      </c>
-      <c r="C93" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C93" t="s">
+        <v>69</v>
       </c>
       <c r="D93" t="s">
         <v>33</v>
@@ -1956,10 +1951,10 @@
         <v>32</v>
       </c>
       <c r="B94" t="s">
-        <v>75</v>
-      </c>
-      <c r="C94" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C94" t="s">
+        <v>69</v>
       </c>
       <c r="D94" t="s">
         <v>16</v>
@@ -1970,10 +1965,10 @@
         <v>49</v>
       </c>
       <c r="B95" t="s">
-        <v>75</v>
-      </c>
-      <c r="C95" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C95" t="s">
+        <v>69</v>
       </c>
       <c r="D95" t="s">
         <v>5</v>
@@ -1984,10 +1979,10 @@
         <v>32</v>
       </c>
       <c r="B96" t="s">
-        <v>75</v>
-      </c>
-      <c r="C96" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C96" t="s">
+        <v>69</v>
       </c>
       <c r="D96" t="s">
         <v>16</v>
@@ -1998,10 +1993,10 @@
         <v>52</v>
       </c>
       <c r="B97" t="s">
-        <v>75</v>
-      </c>
-      <c r="C97" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C97" t="s">
+        <v>69</v>
       </c>
       <c r="D97" t="s">
         <v>34</v>
@@ -2012,10 +2007,10 @@
         <v>32</v>
       </c>
       <c r="B98" t="s">
-        <v>75</v>
-      </c>
-      <c r="C98" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C98" t="s">
+        <v>69</v>
       </c>
       <c r="D98" t="s">
         <v>16</v>
@@ -2026,10 +2021,10 @@
         <v>31</v>
       </c>
       <c r="B99" t="s">
-        <v>75</v>
-      </c>
-      <c r="C99" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C99" t="s">
+        <v>69</v>
       </c>
       <c r="D99" t="s">
         <v>33</v>
@@ -2040,10 +2035,10 @@
         <v>32</v>
       </c>
       <c r="B100" t="s">
-        <v>75</v>
-      </c>
-      <c r="C100" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C100" t="s">
+        <v>69</v>
       </c>
       <c r="D100" t="s">
         <v>16</v>
@@ -2054,10 +2049,10 @@
         <v>49</v>
       </c>
       <c r="B101" t="s">
-        <v>75</v>
-      </c>
-      <c r="C101" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C101" t="s">
+        <v>69</v>
       </c>
       <c r="D101" t="s">
         <v>5</v>
@@ -2068,10 +2063,10 @@
         <v>32</v>
       </c>
       <c r="B102" t="s">
-        <v>75</v>
-      </c>
-      <c r="C102" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C102" t="s">
+        <v>69</v>
       </c>
       <c r="D102" t="s">
         <v>16</v>
@@ -2082,10 +2077,10 @@
         <v>53</v>
       </c>
       <c r="B103" t="s">
-        <v>75</v>
-      </c>
-      <c r="C103" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C103" t="s">
+        <v>69</v>
       </c>
       <c r="D103" t="s">
         <v>34</v>
@@ -2096,10 +2091,10 @@
         <v>32</v>
       </c>
       <c r="B104" t="s">
-        <v>75</v>
-      </c>
-      <c r="C104" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C104" t="s">
+        <v>69</v>
       </c>
       <c r="D104" t="s">
         <v>16</v>
@@ -2110,10 +2105,10 @@
         <v>31</v>
       </c>
       <c r="B105" t="s">
-        <v>75</v>
-      </c>
-      <c r="C105" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C105" t="s">
+        <v>69</v>
       </c>
       <c r="D105" t="s">
         <v>33</v>
@@ -2124,10 +2119,10 @@
         <v>32</v>
       </c>
       <c r="B106" t="s">
-        <v>75</v>
-      </c>
-      <c r="C106" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C106" t="s">
+        <v>69</v>
       </c>
       <c r="D106" t="s">
         <v>16</v>
@@ -2138,10 +2133,10 @@
         <v>49</v>
       </c>
       <c r="B107" t="s">
-        <v>75</v>
-      </c>
-      <c r="C107" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C107" t="s">
+        <v>69</v>
       </c>
       <c r="D107" t="s">
         <v>5</v>
@@ -2152,10 +2147,10 @@
         <v>32</v>
       </c>
       <c r="B108" t="s">
-        <v>75</v>
-      </c>
-      <c r="C108" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C108" t="s">
+        <v>69</v>
       </c>
       <c r="D108" t="s">
         <v>16</v>
@@ -2166,10 +2161,10 @@
         <v>54</v>
       </c>
       <c r="B109" t="s">
-        <v>75</v>
-      </c>
-      <c r="C109" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C109" t="s">
+        <v>69</v>
       </c>
       <c r="D109" t="s">
         <v>34</v>
@@ -2180,10 +2175,10 @@
         <v>32</v>
       </c>
       <c r="B110" t="s">
-        <v>75</v>
-      </c>
-      <c r="C110" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C110" t="s">
+        <v>69</v>
       </c>
       <c r="D110" t="s">
         <v>16</v>
@@ -2194,10 +2189,10 @@
         <v>31</v>
       </c>
       <c r="B111" t="s">
-        <v>75</v>
-      </c>
-      <c r="C111" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C111" t="s">
+        <v>69</v>
       </c>
       <c r="D111" t="s">
         <v>33</v>
@@ -2208,10 +2203,10 @@
         <v>32</v>
       </c>
       <c r="B112" t="s">
-        <v>75</v>
-      </c>
-      <c r="C112" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C112" t="s">
+        <v>69</v>
       </c>
       <c r="D112" t="s">
         <v>16</v>
@@ -2222,10 +2217,10 @@
         <v>49</v>
       </c>
       <c r="B113" t="s">
-        <v>75</v>
-      </c>
-      <c r="C113" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C113" t="s">
+        <v>69</v>
       </c>
       <c r="D113" t="s">
         <v>5</v>
@@ -2236,10 +2231,10 @@
         <v>32</v>
       </c>
       <c r="B114" t="s">
-        <v>75</v>
-      </c>
-      <c r="C114" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C114" t="s">
+        <v>69</v>
       </c>
       <c r="D114" t="s">
         <v>16</v>
@@ -2250,10 +2245,10 @@
         <v>55</v>
       </c>
       <c r="B115" t="s">
-        <v>75</v>
-      </c>
-      <c r="C115" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C115" t="s">
+        <v>69</v>
       </c>
       <c r="D115" t="s">
         <v>34</v>
@@ -2264,10 +2259,10 @@
         <v>32</v>
       </c>
       <c r="B116" t="s">
-        <v>75</v>
-      </c>
-      <c r="C116" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C116" t="s">
+        <v>69</v>
       </c>
       <c r="D116" t="s">
         <v>16</v>
@@ -2278,10 +2273,10 @@
         <v>31</v>
       </c>
       <c r="B117" t="s">
-        <v>75</v>
-      </c>
-      <c r="C117" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C117" t="s">
+        <v>69</v>
       </c>
       <c r="D117" t="s">
         <v>33</v>
@@ -2292,10 +2287,10 @@
         <v>32</v>
       </c>
       <c r="B118" t="s">
-        <v>75</v>
-      </c>
-      <c r="C118" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C118" t="s">
+        <v>69</v>
       </c>
       <c r="D118" t="s">
         <v>16</v>
@@ -2306,10 +2301,10 @@
         <v>49</v>
       </c>
       <c r="B119" t="s">
-        <v>75</v>
-      </c>
-      <c r="C119" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C119" t="s">
+        <v>69</v>
       </c>
       <c r="D119" t="s">
         <v>5</v>
@@ -2320,10 +2315,10 @@
         <v>32</v>
       </c>
       <c r="B120" t="s">
-        <v>75</v>
-      </c>
-      <c r="C120" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C120" t="s">
+        <v>69</v>
       </c>
       <c r="D120" t="s">
         <v>16</v>
@@ -2334,10 +2329,10 @@
         <v>56</v>
       </c>
       <c r="B121" t="s">
-        <v>75</v>
-      </c>
-      <c r="C121" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C121" t="s">
+        <v>69</v>
       </c>
       <c r="D121" t="s">
         <v>34</v>
@@ -2348,10 +2343,10 @@
         <v>32</v>
       </c>
       <c r="B122" t="s">
-        <v>75</v>
-      </c>
-      <c r="C122" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C122" t="s">
+        <v>69</v>
       </c>
       <c r="D122" t="s">
         <v>16</v>
@@ -2362,10 +2357,10 @@
         <v>31</v>
       </c>
       <c r="B123" t="s">
-        <v>75</v>
-      </c>
-      <c r="C123" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C123" t="s">
+        <v>69</v>
       </c>
       <c r="D123" t="s">
         <v>33</v>
@@ -2376,10 +2371,10 @@
         <v>32</v>
       </c>
       <c r="B124" t="s">
-        <v>75</v>
-      </c>
-      <c r="C124" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C124" t="s">
+        <v>69</v>
       </c>
       <c r="D124" t="s">
         <v>16</v>
@@ -2390,10 +2385,10 @@
         <v>49</v>
       </c>
       <c r="B125" t="s">
-        <v>75</v>
-      </c>
-      <c r="C125" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C125" t="s">
+        <v>69</v>
       </c>
       <c r="D125" t="s">
         <v>5</v>
@@ -2404,10 +2399,10 @@
         <v>32</v>
       </c>
       <c r="B126" t="s">
-        <v>75</v>
-      </c>
-      <c r="C126" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C126" t="s">
+        <v>69</v>
       </c>
       <c r="D126" t="s">
         <v>16</v>
@@ -2418,10 +2413,10 @@
         <v>57</v>
       </c>
       <c r="B127" t="s">
-        <v>75</v>
-      </c>
-      <c r="C127" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C127" t="s">
+        <v>69</v>
       </c>
       <c r="D127" t="s">
         <v>34</v>

</xml_diff>